<commit_message>
feature: move vendor qualification pack under the Proof section
Y-04 relocates from /yards-integrators/vendor-qualification-pack/ to
/proof/vendor-qualification-pack/ per boss feedback: the vendor pack
belongs alongside certifications and other evidence, not filed under
the Yards section.

Edited via research/RTG_Website_Page_Map.xlsx (Section, URL slug) and
regenerated src/data/pages.ts with `npm run pagemap`, per CLAUDE.md —
never hand-edit pages.ts. childrenOf()/ancestorsOf() are slug-prefix
derived, so the page automatically becomes a Proof-hub child with
correct breadcrumbs; no template or nav code needed changing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RTG_Website/research/RTG_Website_Page_Map.xlsx
+++ b/RTG_Website/research/RTG_Website_Page_Map.xlsx
@@ -442,7 +442,7 @@
         <v>Meta description</v>
       </c>
       <c r="L1" t="str">
-        <v>Len</v>
+        <v>Len_1</v>
       </c>
       <c r="M1" t="str">
         <v>H1</v>
@@ -504,14 +504,12 @@
         <v>Deck Equipment for Research &amp; Survey Vessels | RTG</v>
       </c>
       <c r="J2">
-        <f>LEN(I2)</f>
         <v>50</v>
       </c>
       <c r="K2" t="str">
         <v>Custom winches, launch and recovery systems and deck machinery for research, survey and geotechnical vessels. Designed in the UK, built and tested in the EU.</v>
       </c>
       <c r="L2">
-        <f>LEN(K2)</f>
         <v>157</v>
       </c>
       <c r="M2" t="str">
@@ -574,14 +572,12 @@
         <v>Sectors We Supply | Survey, Geotechnical, Wind | RTG</v>
       </c>
       <c r="J3">
-        <f>LEN(I3)</f>
         <v>52</v>
       </c>
       <c r="K3" t="str">
         <v>RTG deck equipment works across ocean survey, marine geotechnical, offshore wind and cables, seismic, research, subsea and defence. Find your sector.</v>
       </c>
       <c r="L3">
-        <f>LEN(K3)</f>
         <v>149</v>
       </c>
       <c r="M3" t="str">
@@ -644,14 +640,12 @@
         <v>Survey &amp; Hydrographic Winches and LARS | RTG</v>
       </c>
       <c r="J4">
-        <f>LEN(I4)</f>
         <v>44</v>
       </c>
       <c r="K4" t="str">
         <v>Winches and launch and recovery systems for hydrographic and geophysical survey: CTD, side scan, magnetometer, sub-bottom profiler and deep tow, 300 to 4,000 m.</v>
       </c>
       <c r="L4">
-        <f>LEN(K4)</f>
         <v>160</v>
       </c>
       <c r="M4" t="str">
@@ -714,14 +708,12 @@
         <v>Geotechnical Handling Systems &amp; CPT Winches | RTG</v>
       </c>
       <c r="J5">
-        <f>LEN(I5)</f>
         <v>49</v>
       </c>
       <c r="K5" t="str">
         <v>Corer, CPT and vibrocorer handling systems with tension control for seabed sampling. Proven to a 3,000 m working depth on a CPT sampling system.</v>
       </c>
       <c r="L5">
-        <f>LEN(K5)</f>
         <v>144</v>
       </c>
       <c r="M5" t="str">
@@ -784,14 +776,12 @@
         <v>Offshore Wind &amp; Subsea Cable Handling Equipment | RTG</v>
       </c>
       <c r="J6">
-        <f>LEN(I6)</f>
         <v>53</v>
       </c>
       <c r="K6" t="str">
         <v>Site investigation handling, cable tensioners from 5 to 20 tonnes and containerised cable spreads for offshore wind arrays, export cables and interconnectors.</v>
       </c>
       <c r="L6">
-        <f>LEN(K6)</f>
         <v>158</v>
       </c>
       <c r="M6" t="str">
@@ -854,14 +844,12 @@
         <v>Seismic Source and Streamer Handling Systems | RTG</v>
       </c>
       <c r="J7">
-        <f>LEN(I7)</f>
         <v>50</v>
       </c>
       <c r="K7" t="str">
         <v>Seismic winches, source handling and streamer deployment systems for 2D and 3D marine seismic acquisition, designed for continuous duty at sea.</v>
       </c>
       <c r="L7">
-        <f>LEN(K7)</f>
         <v>143</v>
       </c>
       <c r="M7" t="str">
@@ -924,14 +912,12 @@
         <v>Oceanographic Research Winches | CTD &amp; Deep Tow | RTG</v>
       </c>
       <c r="J8">
-        <f>LEN(I8)</f>
         <v>53</v>
       </c>
       <c r="K8" t="str">
         <v>Research winches for CTD, coring and deep tow work, from 300 to 4,000 m, electric or hydraulic, with precise slow-speed control for repeatable casts.</v>
       </c>
       <c r="L8">
-        <f>LEN(K8)</f>
         <v>149</v>
       </c>
       <c r="M8" t="str">
@@ -994,14 +980,12 @@
         <v>ROV LARS, Umbilical Winches &amp; Dive Systems | RTG</v>
       </c>
       <c r="J9">
-        <f>LEN(I9)</f>
         <v>48</v>
       </c>
       <c r="K9" t="str">
         <v>ROV launch and recovery systems, umbilical and tow winches, diver basket handling and man-riding systems built to class and proven under load.</v>
       </c>
       <c r="L9">
-        <f>LEN(K9)</f>
         <v>142</v>
       </c>
       <c r="M9" t="str">
@@ -1064,14 +1048,12 @@
         <v>Deck Handling Equipment for Defence &amp; Government | RTG</v>
       </c>
       <c r="J10">
-        <f>LEN(I10)</f>
         <v>54</v>
       </c>
       <c r="K10" t="str">
         <v>Deck machinery and handling systems for naval, coastguard and government research vessels, built to class with full material and weld traceability.</v>
       </c>
       <c r="L10">
-        <f>LEN(K10)</f>
         <v>147</v>
       </c>
       <c r="M10" t="str">
@@ -1134,14 +1116,12 @@
         <v>Winches, LARS &amp; Deck Machinery | Equipment | RTG</v>
       </c>
       <c r="J11">
-        <f>LEN(I11)</f>
         <v>48</v>
       </c>
       <c r="K11" t="str">
         <v>The RTG equipment range: winches, launch and recovery systems, cranes, handling systems, power units and containerised spreads for survey and subsea work.</v>
       </c>
       <c r="L11">
-        <f>LEN(K11)</f>
         <v>154</v>
       </c>
       <c r="M11" t="str">
@@ -1204,14 +1184,12 @@
         <v>Marine Winches | Survey, Geotechnical &amp; ROV | RTG</v>
       </c>
       <c r="J12">
-        <f>LEN(I12)</f>
         <v>49</v>
       </c>
       <c r="K12" t="str">
         <v>Electric and hydraulic marine winches from 0.3 to 7.4 tonnes working load and 200 to 5,500 m capacity, with Lebus grooved drums and controlled level wind.</v>
       </c>
       <c r="L12">
-        <f>LEN(K12)</f>
         <v>154</v>
       </c>
       <c r="M12" t="str">
@@ -1274,14 +1252,12 @@
         <v>Geotechnical &amp; Coring Winches | CPT &amp; Piston Corer | RTG</v>
       </c>
       <c r="J13">
-        <f>LEN(I13)</f>
         <v>56</v>
       </c>
       <c r="K13" t="str">
         <v>Winches for piston, gravity and box coring and CPT deployment, with constant tension control to protect the umbilical when the tool is captive in the seabed.</v>
       </c>
       <c r="L13">
-        <f>LEN(K13)</f>
         <v>157</v>
       </c>
       <c r="M13" t="str">
@@ -1344,14 +1320,12 @@
         <v>Survey &amp; Oceanographic Winches | 300-4,000 m | RTG</v>
       </c>
       <c r="J14">
-        <f>LEN(I14)</f>
         <v>50</v>
       </c>
       <c r="K14" t="str">
         <v>Survey and oceanographic winches in electric or hydraulic drive, with or without level wind, supplied with cable capacities from 300 to 4,000 metres.</v>
       </c>
       <c r="L14">
-        <f>LEN(K14)</f>
         <v>149</v>
       </c>
       <c r="M14" t="str">
@@ -1414,14 +1388,12 @@
         <v>Seismic Winches &amp; Source Handling | RTG</v>
       </c>
       <c r="J15">
-        <f>LEN(I15)</f>
         <v>39</v>
       </c>
       <c r="K15" t="str">
         <v>Seismic winches and source handling equipment engineered for continuous duty, high line speeds and repeated deployment cycles in marine acquisition.</v>
       </c>
       <c r="L15">
-        <f>LEN(K15)</f>
         <v>148</v>
       </c>
       <c r="M15" t="str">
@@ -1484,14 +1456,12 @@
         <v>ROV, Tow &amp; Umbilical Winches | Slip Ring Ready | RTG</v>
       </c>
       <c r="J16">
-        <f>LEN(I16)</f>
         <v>52</v>
       </c>
       <c r="K16" t="str">
         <v>ROV, deep tow and umbilical winches with Lebus grooved drums, controlled level wind and a slip ring interface to suit your own data and power architecture.</v>
       </c>
       <c r="L16">
-        <f>LEN(K16)</f>
         <v>155</v>
       </c>
       <c r="M16" t="str">
@@ -1554,14 +1524,12 @@
         <v>Mooring &amp; Utility Winches for Offshore Vessels | RTG</v>
       </c>
       <c r="J17">
-        <f>LEN(I17)</f>
         <v>52</v>
       </c>
       <c r="K17" t="str">
         <v>Mooring, capstan and general utility winches for offshore and research vessels, built to class with the same welding and test discipline as the survey range.</v>
       </c>
       <c r="L17">
-        <f>LEN(K17)</f>
         <v>157</v>
       </c>
       <c r="M17" t="str">
@@ -1624,14 +1592,12 @@
         <v>Launch and Recovery Systems | A-Frames &amp; LARS | RTG</v>
       </c>
       <c r="J18">
-        <f>LEN(I18)</f>
         <v>51</v>
       </c>
       <c r="K18" t="str">
         <v>Stern and side A-frames, mini survey LARS, ROV and CTD launch and recovery systems, engineered around your deck arrangement and sea state requirement.</v>
       </c>
       <c r="L18">
-        <f>LEN(K18)</f>
         <v>150</v>
       </c>
       <c r="M18" t="str">
@@ -1694,14 +1660,12 @@
         <v>Marine Cranes &amp; Lifting Equipment | Class Certified | RTG</v>
       </c>
       <c r="J19">
-        <f>LEN(I19)</f>
         <v>57</v>
       </c>
       <c r="K19" t="str">
         <v>Deck cranes, knuckle boom and telescopic lifting equipment for research and offshore vessels, class certified and proof tested before dispatch.</v>
       </c>
       <c r="L19">
-        <f>LEN(K19)</f>
         <v>143</v>
       </c>
       <c r="M19" t="str">
@@ -1764,14 +1728,12 @@
         <v>Corer, Seismic &amp; Cable Handling Systems | RTG</v>
       </c>
       <c r="J20">
-        <f>LEN(I20)</f>
         <v>45</v>
       </c>
       <c r="K20" t="str">
         <v>Complete handling systems for corers, seismic sources, diver baskets and subsea cable, supplied as integrated deck spreads rather than individual machines.</v>
       </c>
       <c r="L20">
-        <f>LEN(K20)</f>
         <v>155</v>
       </c>
       <c r="M20" t="str">
@@ -1834,14 +1796,12 @@
         <v>Cable &amp; Pipe Tensioners | 5 to 20 Te | RTG</v>
       </c>
       <c r="J21">
-        <f>LEN(I21)</f>
         <v>42</v>
       </c>
       <c r="K21" t="str">
         <v>Self-contained two-track electro-hydraulic tensioners from 5 to 20 tonnes on a common skid, remote console controlled, for cable and pipe laying operations.</v>
       </c>
       <c r="L21">
-        <f>LEN(K21)</f>
         <v>156</v>
       </c>
       <c r="M21" t="str">
@@ -1904,14 +1864,12 @@
         <v>Marine Hydraulic Power Units | HPU | RTG</v>
       </c>
       <c r="J22">
-        <f>LEN(I22)</f>
         <v>40</v>
       </c>
       <c r="K22" t="str">
         <v>Hydraulic power units for deck machinery, built and flushed to a defined cleanliness class and function tested with the equipment they will drive.</v>
       </c>
       <c r="L22">
-        <f>LEN(K22)</f>
         <v>146</v>
       </c>
       <c r="M22" t="str">
@@ -1974,14 +1932,12 @@
         <v>Containerised &amp; Portable Survey Spreads | RTG</v>
       </c>
       <c r="J23">
-        <f>LEN(I23)</f>
         <v>45</v>
       </c>
       <c r="K23" t="str">
         <v>Self-contained, road transportable handling spreads with certified lifting lugs, fork pockets and twist-lock footprints, for vessels you do not own.</v>
       </c>
       <c r="L23">
-        <f>LEN(K23)</f>
         <v>148</v>
       </c>
       <c r="M23" t="str">
@@ -2044,14 +2000,12 @@
         <v>Refurbishment, Upgrade &amp; Support | Lifecycle | RTG</v>
       </c>
       <c r="J24">
-        <f>LEN(I24)</f>
         <v>50</v>
       </c>
       <c r="K24" t="str">
         <v>Your vessel is worth more working than replaced. Condition assessment, refurbishment, capability upgrade, re-certification and spares for deck machinery.</v>
       </c>
       <c r="L24">
-        <f>LEN(K24)</f>
         <v>153</v>
       </c>
       <c r="M24" t="str">
@@ -2114,14 +2068,12 @@
         <v>Winch &amp; LARS Refurbishment and Upgrade | RTG</v>
       </c>
       <c r="J25">
-        <f>LEN(I25)</f>
         <v>44</v>
       </c>
       <c r="K25" t="str">
         <v>Full refurbishment of winches, LARS and deck machinery: condition assessment, rework, component reuse, capability upgrade, testing and reissued documentation.</v>
       </c>
       <c r="L25">
-        <f>LEN(K25)</f>
         <v>158</v>
       </c>
       <c r="M25" t="str">
@@ -2184,14 +2136,12 @@
         <v>Refurbish, Upgrade or Replace? A Decision Guide | RTG</v>
       </c>
       <c r="J26">
-        <f>LEN(I26)</f>
         <v>53</v>
       </c>
       <c r="K26" t="str">
         <v>Six questions that decide whether deck machinery is worth rebuilding: drum and shaft condition, brakes, hydraulics, capability target, spares and class status.</v>
       </c>
       <c r="L26">
-        <f>LEN(K26)</f>
         <v>159</v>
       </c>
       <c r="M26" t="str">
@@ -2254,14 +2204,12 @@
         <v>Deck Equipment Re-certification &amp; Class Renewal | RTG</v>
       </c>
       <c r="J27">
-        <f>LEN(I27)</f>
         <v>53</v>
       </c>
       <c r="K27" t="str">
         <v>Load testing, inspection and documentation for class renewal on deck machinery, including equipment originally supplied by other manufacturers.</v>
       </c>
       <c r="L27">
-        <f>LEN(K27)</f>
         <v>143</v>
       </c>
       <c r="M27" t="str">
@@ -2324,14 +2272,12 @@
         <v>Marine Deck Machinery Spares &amp; Support | RTG</v>
       </c>
       <c r="J28">
-        <f>LEN(I28)</f>
         <v>44</v>
       </c>
       <c r="K28" t="str">
         <v>Spares, technical support and field service for RTG equipment and for deck machinery supplied by others, through UK and EU offices and agents worldwide.</v>
       </c>
       <c r="L28">
-        <f>LEN(K28)</f>
         <v>152</v>
       </c>
       <c r="M28" t="str">
@@ -2394,14 +2340,12 @@
         <v>Book a Deck Machinery Condition Assessment | RTG</v>
       </c>
       <c r="J29">
-        <f>LEN(I29)</f>
         <v>48</v>
       </c>
       <c r="K29" t="str">
         <v>Tell us the equipment, the vessel and the maintenance window. We will tell you what is worth rebuilding, what is not, and what the work would involve.</v>
       </c>
       <c r="L29">
-        <f>LEN(K29)</f>
         <v>150</v>
       </c>
       <c r="M29" t="str">
@@ -2464,14 +2408,12 @@
         <v>Contract Manufacturing to Your Drawings | RTG</v>
       </c>
       <c r="J30">
-        <f>LEN(I30)</f>
         <v>45</v>
       </c>
       <c r="K30" t="str">
         <v>Your design, your IP, our factory. From welded structures to complete machines, assembled, piped, wired, programmed, load tested under class and commissioned.</v>
       </c>
       <c r="L30">
-        <f>LEN(K30)</f>
         <v>158</v>
       </c>
       <c r="M30" t="str">
@@ -2534,14 +2476,12 @@
         <v>Certified Structural Fabrication &amp; Welding | RTG</v>
       </c>
       <c r="J31">
-        <f>LEN(I31)</f>
         <v>48</v>
       </c>
       <c r="K31" t="str">
         <v>Welded structures to your drawings with EN ISO 3834 discipline, coded welders, NDT to ISO 9712 level 2 and 100 percent traceability on structural welds.</v>
       </c>
       <c r="L31">
-        <f>LEN(K31)</f>
         <v>152</v>
       </c>
       <c r="M31" t="str">
@@ -2604,14 +2544,12 @@
         <v>Mechanical Assembly to Client Drawings | RTG</v>
       </c>
       <c r="J32">
-        <f>LEN(I32)</f>
         <v>44</v>
       </c>
       <c r="K32" t="str">
         <v>Drums, shafts, bearings, gearboxes, brakes, sheaves and level wind assembled to your specification, torqued, aligned and rotation checked before dispatch.</v>
       </c>
       <c r="L32">
-        <f>LEN(K32)</f>
         <v>154</v>
       </c>
       <c r="M32" t="str">
@@ -2674,14 +2612,12 @@
         <v>Hydraulic &amp; Electrical Build to Your Design | RTG</v>
       </c>
       <c r="J33">
-        <f>LEN(I33)</f>
         <v>49</v>
       </c>
       <c r="K33" t="str">
         <v>Power units, pipework flushed to a defined cleanliness class, valve blocks, control panels, cabling, terminations and instrumentation, built to your schematics.</v>
       </c>
       <c r="L33">
-        <f>LEN(K33)</f>
         <v>160</v>
       </c>
       <c r="M33" t="str">
@@ -2744,14 +2680,12 @@
         <v>Automation, Load Testing &amp; Commissioning | RTG</v>
       </c>
       <c r="J34">
-        <f>LEN(I34)</f>
         <v>46</v>
       </c>
       <c r="K34" t="str">
         <v>PLC and HMI loading, interlock proving, load testing to 150 tonnes under class witness, full certification dossier and commissioning on the vessel.</v>
       </c>
       <c r="L34">
-        <f>LEN(K34)</f>
         <v>147</v>
       </c>
       <c r="M34" t="str">
@@ -2814,14 +2748,12 @@
         <v>Bespoke Deck Equipment Design &amp; Build | RTG</v>
       </c>
       <c r="J35">
-        <f>LEN(I35)</f>
         <v>43</v>
       </c>
       <c r="K35" t="str">
         <v>Where you do not hold a design, RTG engineers one: concept, general arrangement, calculations, class appraisal, manufacture and test, to your requirement.</v>
       </c>
       <c r="L35">
-        <f>LEN(K35)</f>
         <v>154</v>
       </c>
       <c r="M35" t="str">
@@ -2884,14 +2816,12 @@
         <v>How We Protect Your Design and IP | RTG</v>
       </c>
       <c r="J36">
-        <f>LEN(I36)</f>
         <v>39</v>
       </c>
       <c r="K36" t="str">
         <v>NDA before drawings, segregated project files, no derivative products from client designs, and a clear contractual separation from our own equipment range.</v>
       </c>
       <c r="L36">
-        <f>LEN(K36)</f>
         <v>155</v>
       </c>
       <c r="M36" t="str">
@@ -2954,14 +2884,12 @@
         <v>EU-Origin Steel Fabrication &amp; Melt-and-Pour | RTG</v>
       </c>
       <c r="J37">
-        <f>LEN(I37)</f>
         <v>49</v>
       </c>
       <c r="K37" t="str">
         <v>Fabrication inside the EU, with melt-and-pour origin documentation supplied alongside our standard weld traceability pack for every structure we build.</v>
       </c>
       <c r="L37">
-        <f>LEN(K37)</f>
         <v>151</v>
       </c>
       <c r="M37" t="str">
@@ -3024,14 +2952,12 @@
         <v>Current Manufacturing Capacity &amp; Lead Times | RTG</v>
       </c>
       <c r="J38">
-        <f>LEN(I38)</f>
         <v>49</v>
       </c>
       <c r="K38" t="str">
         <v>A quarterly statement of available fabrication, assembly, hydraulic build and test capacity by tier, with indicative lead times for each. Updated every quarter.</v>
       </c>
       <c r="L38">
-        <f>LEN(K38)</f>
         <v>160</v>
       </c>
       <c r="M38" t="str">
@@ -3094,14 +3020,12 @@
         <v>Send Us Your Drawings, Under NDA | RTG</v>
       </c>
       <c r="J39">
-        <f>LEN(I39)</f>
         <v>38</v>
       </c>
       <c r="K39" t="str">
         <v>Upload your documentation under NDA and we will come back with scope, tier options and an indicative price. Tell us which tier you are short of capacity in.</v>
       </c>
       <c r="L39">
-        <f>LEN(K39)</f>
         <v>156</v>
       </c>
       <c r="M39" t="str">
@@ -3164,14 +3088,12 @@
         <v>Subcontract Fabrication &amp; Deck Packages for Yards | RTG</v>
       </c>
       <c r="J40">
-        <f>LEN(I40)</f>
         <v>55</v>
       </c>
       <c r="K40" t="str">
         <v>European standards, EU capacity, class certified. Overflow structural fabrication and deck equipment packages that protect your delivery date.</v>
       </c>
       <c r="L40">
-        <f>LEN(K40)</f>
         <v>142</v>
       </c>
       <c r="M40" t="str">
@@ -3234,14 +3156,12 @@
         <v>Structural Steel Subcontracting for Shipyards | RTG</v>
       </c>
       <c r="J41">
-        <f>LEN(I41)</f>
         <v>51</v>
       </c>
       <c r="K41" t="str">
         <v>Overflow structural fabrication, sea-fastenings and large welded assemblies, class surveyed, delivered to your build programme from an EU facility.</v>
       </c>
       <c r="L41">
-        <f>LEN(K41)</f>
         <v>147</v>
       </c>
       <c r="M41" t="str">
@@ -3304,14 +3224,12 @@
         <v>Deck Equipment Packages for Newbuild Vessels | RTG</v>
       </c>
       <c r="J42">
-        <f>LEN(I42)</f>
         <v>50</v>
       </c>
       <c r="K42" t="str">
         <v>Complete deck handling packages specified, built, tested and commissioned for newbuild survey, research and offshore vessels, integrated with your programme.</v>
       </c>
       <c r="L42">
-        <f>LEN(K42)</f>
         <v>157</v>
       </c>
       <c r="M42" t="str">
@@ -3374,14 +3292,12 @@
         <v>Certifications, Class Approvals &amp; Welding Standards | RTG</v>
       </c>
       <c r="J43">
-        <f>LEN(I43)</f>
         <v>57</v>
       </c>
       <c r="K43" t="str">
         <v>Bureau Veritas Mode II recognition, welding procedures approved with TUV, DNV and Lloyd's Register, welders to ISO 9606-1 and NDT to ISO 9712 level 2.</v>
       </c>
       <c r="L43">
-        <f>LEN(K43)</f>
         <v>150</v>
       </c>
       <c r="M43" t="str">
@@ -3420,13 +3336,13 @@
         <v>Y-04</v>
       </c>
       <c r="B44" t="str">
-        <v>Yards</v>
+        <v>Proof</v>
       </c>
       <c r="C44" t="str">
         <v>Vendor Qualification Pack</v>
       </c>
       <c r="D44" t="str">
-        <v>/yards-integrators/vendor-qualification-pack/</v>
+        <v>/proof/vendor-qualification-pack/</v>
       </c>
       <c r="E44" t="str">
         <v>Form</v>
@@ -3444,14 +3360,12 @@
         <v>Download Our Vendor Qualification Pack | RTG</v>
       </c>
       <c r="J44">
-        <f>LEN(I44)</f>
         <v>44</v>
       </c>
       <c r="K44" t="str">
         <v>Everything your procurement and quality teams need to assess RTG as an approved fabricator, in one document. Tell us the yard and the programme it is for.</v>
       </c>
       <c r="L44">
-        <f>LEN(K44)</f>
         <v>154</v>
       </c>
       <c r="M44" t="str">
@@ -3514,14 +3428,12 @@
         <v>Case Studies, References &amp; Test Evidence | RTG</v>
       </c>
       <c r="J45">
-        <f>LEN(I45)</f>
         <v>46</v>
       </c>
       <c r="K45" t="str">
         <v>Twenty-two years, more than 250 completed projects and around 1,500 deck machines. Case studies, vessel references, our test facility and what clients say.</v>
       </c>
       <c r="L45">
-        <f>LEN(K45)</f>
         <v>155</v>
       </c>
       <c r="M45" t="str">
@@ -3584,14 +3496,12 @@
         <v>Deck Equipment Case Studies | RTG</v>
       </c>
       <c r="J46">
-        <f>LEN(I46)</f>
         <v>33</v>
       </c>
       <c r="K46" t="str">
         <v>How RTG standardised handling across a survey fleet, rebuilt a twelve-year-old traction winch, and built complete machines to an OEM's drawings.</v>
       </c>
       <c r="L46">
-        <f>LEN(K46)</f>
         <v>144</v>
       </c>
       <c r="M46" t="str">
@@ -3654,14 +3564,12 @@
         <v>Case Study: One Handling Standard, Seven Vessels | RTG</v>
       </c>
       <c r="J47">
-        <f>LEN(I47)</f>
         <v>54</v>
       </c>
       <c r="K47" t="str">
         <v>How a survey operator moved from a patchwork of launch and recovery systems to a single handling standard across seven vessels over fourteen years.</v>
       </c>
       <c r="L47">
-        <f>LEN(K47)</f>
         <v>147</v>
       </c>
       <c r="M47" t="str">
@@ -3724,14 +3632,12 @@
         <v>Case Study: Rebuilding a 2009 Traction Winch | RTG</v>
       </c>
       <c r="J48">
-        <f>LEN(I48)</f>
         <v>50</v>
       </c>
       <c r="K48" t="str">
         <v>A twelve-year-old electro-hydraulic traction winch assessed, rebuilt, upgraded and retested for offshore geotechnical work, with documentation reissued.</v>
       </c>
       <c r="L48">
-        <f>LEN(K48)</f>
         <v>152</v>
       </c>
       <c r="M48" t="str">
@@ -3794,14 +3700,12 @@
         <v>Case Study: A Complete Machine, Built to Their Drawings</v>
       </c>
       <c r="J49">
-        <f>LEN(I49)</f>
         <v>55</v>
       </c>
       <c r="K49" t="str">
         <v>How an equipment OEM moved from outsourcing steelwork alone to handing RTG a complete machine, assembled, wired, tested under class and delivered.</v>
       </c>
       <c r="L49">
-        <f>LEN(K49)</f>
         <v>146</v>
       </c>
       <c r="M49" t="str">
@@ -3864,14 +3768,12 @@
         <v>Case Study: Deck Equipment for a Newbuild Programme | RTG</v>
       </c>
       <c r="J50">
-        <f>LEN(I50)</f>
         <v>57</v>
       </c>
       <c r="K50" t="str">
         <v>Supplying and commissioning deck handling equipment into a shipyard newbuild programme, delivered to the yard's own schedule and certified to class throughout.</v>
       </c>
       <c r="L50">
-        <f>LEN(K50)</f>
         <v>159</v>
       </c>
       <c r="M50" t="str">
@@ -3934,14 +3836,12 @@
         <v>Load Testing to 150 Tonnes | Test Facility | RTG</v>
       </c>
       <c r="J51">
-        <f>LEN(I51)</f>
         <v>48</v>
       </c>
       <c r="K51" t="str">
         <v>Two test stands, load testing to 150 tonnes with certified weights: proof load, dynamic functional, brake holding, render and speed tests under class witness.</v>
       </c>
       <c r="L51">
-        <f>LEN(K51)</f>
         <v>158</v>
       </c>
       <c r="M51" t="str">
@@ -4004,14 +3904,12 @@
         <v>Vessels and Clients We Have Supplied | RTG</v>
       </c>
       <c r="J52">
-        <f>LEN(I52)</f>
         <v>42</v>
       </c>
       <c r="K52" t="str">
         <v>More than 50 global customers and research institutions, over 250 completed projects and around 1,500 custom deck machines delivered since 2003.</v>
       </c>
       <c r="L52">
-        <f>LEN(K52)</f>
         <v>144</v>
       </c>
       <c r="M52" t="str">
@@ -4074,14 +3972,12 @@
         <v>What Our Clients Say | Testimonials | RTG</v>
       </c>
       <c r="J53">
-        <f>LEN(I53)</f>
         <v>41</v>
       </c>
       <c r="K53" t="str">
         <v>In the words of a global survey operator, a major shipyard and an offshore equipment specialist, on design quality, communication and on-time delivery.</v>
       </c>
       <c r="L53">
-        <f>LEN(K53)</f>
         <v>151</v>
       </c>
       <c r="M53" t="str">
@@ -4144,14 +4040,12 @@
         <v>Technical Notes on Deck Machinery Engineering | RTG</v>
       </c>
       <c r="J54">
-        <f>LEN(I54)</f>
         <v>51</v>
       </c>
       <c r="K54" t="str">
         <v>Plain explanations of how deck machinery works: layer effect on line pull, Lebus grooving, lead-off angle, render testing, squeeze versus line tension.</v>
       </c>
       <c r="L54">
-        <f>LEN(K54)</f>
         <v>151</v>
       </c>
       <c r="M54" t="str">
@@ -4214,14 +4108,12 @@
         <v>Request Equipment Datasheets | RTG</v>
       </c>
       <c r="J55">
-        <f>LEN(I55)</f>
         <v>34</v>
       </c>
       <c r="K55" t="str">
         <v>Full datasheets including general arrangement drawings, issued to you by email. Tell us the equipment and the project and we will send the right ones.</v>
       </c>
       <c r="L55">
-        <f>LEN(K55)</f>
         <v>150</v>
       </c>
       <c r="M55" t="str">
@@ -4284,14 +4176,12 @@
         <v>Product Catalogues | RTG</v>
       </c>
       <c r="J56">
-        <f>LEN(I56)</f>
         <v>24</v>
       </c>
       <c r="K56" t="str">
         <v>The full RTG deck equipment catalogue, issued on request. Tell us your sector and the work you do and we will send you the relevant volume by email.</v>
       </c>
       <c r="L56">
-        <f>LEN(K56)</f>
         <v>148</v>
       </c>
       <c r="M56" t="str">
@@ -4354,14 +4244,12 @@
         <v>News and Insight | RTG</v>
       </c>
       <c r="J57">
-        <f>LEN(I57)</f>
         <v>22</v>
       </c>
       <c r="K57" t="str">
         <v>Project news, technical insight and market commentary on deck machinery and offshore handling, from RTG's UK and Romanian engineering teams. Updated monthly.</v>
       </c>
       <c r="L57">
-        <f>LEN(K57)</f>
         <v>157</v>
       </c>
       <c r="M57" t="str">
@@ -4424,14 +4312,12 @@
         <v>About RTG | British Design, European Manufacture</v>
       </c>
       <c r="J58">
-        <f>LEN(I58)</f>
         <v>48</v>
       </c>
       <c r="K58" t="str">
         <v>Founded to combine British deck equipment design with European manufacturing. Twenty-two years, 250 projects and around 1,500 machines delivered.</v>
       </c>
       <c r="L58">
-        <f>LEN(K58)</f>
         <v>145</v>
       </c>
       <c r="M58" t="str">
@@ -4494,14 +4380,12 @@
         <v>Our People and Our Factory at Satu Mare | RTG</v>
       </c>
       <c r="J59">
-        <f>LEN(I59)</f>
         <v>45</v>
       </c>
       <c r="K59" t="str">
         <v>Around 80 engineers, welders, fitters and technicians in a purpose-built facility in Satu Mare, Romania, with design and commercial teams in the UK.</v>
       </c>
       <c r="L59">
-        <f>LEN(K59)</f>
         <v>148</v>
       </c>
       <c r="M59" t="str">
@@ -4564,14 +4448,12 @@
         <v>Quality, Health, Safety and Environment | RTG</v>
       </c>
       <c r="J60">
-        <f>LEN(I60)</f>
         <v>45</v>
       </c>
       <c r="K60" t="str">
         <v>How RTG manages quality, safety and environmental responsibility across design, manufacture, testing and site work, and the standards it is assessed against.</v>
       </c>
       <c r="L60">
-        <f>LEN(K60)</f>
         <v>157</v>
       </c>
       <c r="M60" t="str">
@@ -4634,14 +4516,12 @@
         <v>Sustainability and Ocean Research | RTG</v>
       </c>
       <c r="J61">
-        <f>LEN(I61)</f>
         <v>39</v>
       </c>
       <c r="K61" t="str">
         <v>Equipment designed for long service life and refurbishment rather than replacement, supporting ocean research and offshore renewable energy.</v>
       </c>
       <c r="L61">
-        <f>LEN(K61)</f>
         <v>140</v>
       </c>
       <c r="M61" t="str">
@@ -4704,14 +4584,12 @@
         <v>Careers at RTG | Engineering Jobs in Satu Mare and the UK</v>
       </c>
       <c r="J62">
-        <f>LEN(I62)</f>
         <v>57</v>
       </c>
       <c r="K62" t="str">
         <v>Welding, mechanical, hydraulic, electrical, automation and design roles in Satu Mare and the UK. See what we build and who you would build it with.</v>
       </c>
       <c r="L62">
-        <f>LEN(K62)</f>
         <v>147</v>
       </c>
       <c r="M62" t="str">
@@ -4774,14 +4652,12 @@
         <v>Contact RTG | UK and Romania Offices</v>
       </c>
       <c r="J63">
-        <f>LEN(I63)</f>
         <v>36</v>
       </c>
       <c r="K63" t="str">
         <v>Talk to our UK commercial team or our factory at Satu Mare in Romania, or find your regional agent across the Americas and Asia Pacific. We answer quickly.</v>
       </c>
       <c r="L63">
-        <f>LEN(K63)</f>
         <v>155</v>
       </c>
       <c r="M63" t="str">
@@ -4844,14 +4720,12 @@
         <v>Our Agents in the Americas and Asia Pacific | RTG</v>
       </c>
       <c r="J64">
-        <f>LEN(I64)</f>
         <v>49</v>
       </c>
       <c r="K64" t="str">
         <v>Local representation for sales, support and spares across the Americas and Asia Pacific, backed directly by the engineers who designed and built the equipment.</v>
       </c>
       <c r="L64">
-        <f>LEN(K64)</f>
         <v>159</v>
       </c>
       <c r="M64" t="str">
@@ -4914,14 +4788,12 @@
         <v>Request a Quotation | RTG</v>
       </c>
       <c r="J65">
-        <f>LEN(I65)</f>
         <v>25</v>
       </c>
       <c r="K65" t="str">
         <v>Tell us the duty, the vessel and the timescale. We will come back with a proposed configuration and an indicative price, and say what we still need.</v>
       </c>
       <c r="L65">
-        <f>LEN(K65)</f>
         <v>148</v>
       </c>
       <c r="M65" t="str">
@@ -4984,14 +4856,12 @@
         <v>Aftersales, Spares and Field Service | RTG</v>
       </c>
       <c r="J66">
-        <f>LEN(I66)</f>
         <v>42</v>
       </c>
       <c r="K66" t="str">
         <v>Existing equipment, urgent spares or a technical problem at sea. Tell us the equipment and the vessel and we will route it to the right engineer.</v>
       </c>
       <c r="L66">
-        <f>LEN(K66)</f>
         <v>145</v>
       </c>
       <c r="M66" t="str">
@@ -5054,14 +4924,12 @@
         <v>Privacy Notice | RTG</v>
       </c>
       <c r="J67">
-        <f>LEN(I67)</f>
         <v>20</v>
       </c>
       <c r="K67" t="str">
         <v>How RTG collects, uses and stores personal data submitted through this website, and your rights under UK and EU data protection law.</v>
       </c>
       <c r="L67">
-        <f>LEN(K67)</f>
         <v>132</v>
       </c>
       <c r="M67" t="str">
@@ -5124,14 +4992,12 @@
         <v>Cookie Policy | RTG</v>
       </c>
       <c r="J68">
-        <f>LEN(I68)</f>
         <v>19</v>
       </c>
       <c r="K68" t="str">
         <v>The cookies and similar technologies used on this website, what each is for, and how to change your consent at any time.</v>
       </c>
       <c r="L68">
-        <f>LEN(K68)</f>
         <v>120</v>
       </c>
       <c r="M68" t="str">
@@ -5194,14 +5060,12 @@
         <v>Terms of Use and Copyright | RTG</v>
       </c>
       <c r="J69">
-        <f>LEN(I69)</f>
         <v>32</v>
       </c>
       <c r="K69" t="str">
         <v>Terms governing use of this website and of documentation issued through it, including copyright in RTG drawings and technical publications.</v>
       </c>
       <c r="L69">
-        <f>LEN(K69)</f>
         <v>139</v>
       </c>
       <c r="M69" t="str">
@@ -5264,14 +5128,12 @@
         <v>Accessibility Statement | RTG</v>
       </c>
       <c r="J70">
-        <f>LEN(I70)</f>
         <v>29</v>
       </c>
       <c r="K70" t="str">
         <v>How this website is designed to be usable by everyone, the standard it targets, and how to report a problem.</v>
       </c>
       <c r="L70">
-        <f>LEN(K70)</f>
         <v>108</v>
       </c>
       <c r="M70" t="str">
@@ -5334,14 +5196,12 @@
         <v>Resources | Datasheets, Notes &amp; News | RTG</v>
       </c>
       <c r="J71">
-        <f>LEN(I71)</f>
         <v>42</v>
       </c>
       <c r="K71" t="str">
         <v>Technical notes, open datasheets, catalogues and industry news for engineers specifying deck equipment — everything RTG publishes, gathered in one place.</v>
       </c>
       <c r="L71">
-        <f>LEN(K71)</f>
         <v>153</v>
       </c>
       <c r="M71" t="str">
@@ -5380,14 +5240,12 @@
         <v>TOTALS</v>
       </c>
       <c r="H72">
-        <f>COUNTIF(H2:H70,"P1")</f>
         <v>47</v>
       </c>
       <c r="I72" t="str">
         <v>P1 pages</v>
       </c>
       <c r="T72">
-        <f>SUM(T2:T70)</f>
         <v>39200</v>
       </c>
       <c r="U72" t="str">
@@ -5396,14 +5254,12 @@
     </row>
     <row r="73">
       <c r="I73">
-        <f>COUNTIF(J2:J70,"&gt;60")</f>
         <v>0</v>
       </c>
       <c r="K73" t="str">
         <v>title tags over 60 chars - fix these</v>
       </c>
       <c r="L73">
-        <f>COUNTIF(L2:L70,"&gt;160")</f>
         <v>0</v>
       </c>
       <c r="M73" t="str">
@@ -5411,8 +5267,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V70"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:V73"/>
   </ignoredErrors>

</xml_diff>